<commit_message>
data and figures added
</commit_message>
<xml_diff>
--- a/SI_Table_1.xlsx
+++ b/SI_Table_1.xlsx
@@ -761,7 +761,7 @@
         <v>0.35</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>27</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>0.13</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29">
@@ -841,7 +841,7 @@
         <v>0.35</v>
       </c>
       <c r="F31" t="s" s="0">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">

</xml_diff>